<commit_message>
Correct October 26 Daytona prices
Co-authored-by: DanielWang2029 <DanielWang2029@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/output/gpu_prices_20261026.xlsx
+++ b/output/gpu_prices_20261026.xlsx
@@ -129,8 +129,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="DailyGpuPrices" displayName="DailyGpuPrices" ref="A1:G94" headerRowCount="1">
-  <autoFilter ref="A1:G94"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="DailyGpuPrices" displayName="DailyGpuPrices" ref="A1:G92" headerRowCount="1">
+  <autoFilter ref="A1:G92"/>
   <tableColumns count="7">
     <tableColumn id="1" name="dtstatdate"/>
     <tableColumn id="2" name="source_name"/>
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G94"/>
+  <dimension ref="A1:G92"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1109,7 +1109,7 @@
         </is>
       </c>
       <c r="G19" t="n">
-        <v>3</v>
+        <v>2.7</v>
       </c>
     </row>
     <row r="20">
@@ -1179,7 +1179,7 @@
         </is>
       </c>
       <c r="G21" t="n">
-        <v>5.39</v>
+        <v>5.09</v>
       </c>
     </row>
     <row r="22">
@@ -2194,7 +2194,7 @@
         </is>
       </c>
       <c r="G50" t="n">
-        <v>6.25</v>
+        <v>7.1</v>
       </c>
     </row>
     <row r="51">
@@ -2333,6 +2333,9 @@
           <t>N/A</t>
         </is>
       </c>
+      <c r="G54" t="n">
+        <v>4.54</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -2365,6 +2368,9 @@
           <t>N/A</t>
         </is>
       </c>
+      <c r="G55" t="n">
+        <v>2.61</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -2519,7 +2525,7 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>B300</t>
+          <t>B200</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
@@ -2536,6 +2542,9 @@
         <is>
           <t>N/A</t>
         </is>
+      </c>
+      <c r="G60" t="n">
+        <v>7.99</v>
       </c>
     </row>
     <row r="61">
@@ -2551,7 +2560,7 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>B200</t>
+          <t>H200</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -2570,7 +2579,7 @@
         </is>
       </c>
       <c r="G61" t="n">
-        <v>7.99</v>
+        <v>5.29</v>
       </c>
     </row>
     <row r="62">
@@ -2586,7 +2595,7 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>H200</t>
+          <t>A100</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -2605,7 +2614,7 @@
         </is>
       </c>
       <c r="G62" t="n">
-        <v>5.29</v>
+        <v>1.07</v>
       </c>
     </row>
     <row r="63">
@@ -2616,17 +2625,17 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Gpu.ai</t>
+          <t>Spheron</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>A100</t>
+          <t>B300</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>On-Demand</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -2640,7 +2649,7 @@
         </is>
       </c>
       <c r="G63" t="n">
-        <v>1.07</v>
+        <v>12.42</v>
       </c>
     </row>
     <row r="64">
@@ -2661,7 +2670,7 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>On-Demand</t>
+          <t>Spot</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
@@ -2675,7 +2684,7 @@
         </is>
       </c>
       <c r="G64" t="n">
-        <v>12.42</v>
+        <v>5.84</v>
       </c>
     </row>
     <row r="65">
@@ -2691,12 +2700,12 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>B300</t>
+          <t>B200</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Spot</t>
+          <t>On-Demand</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
@@ -2710,7 +2719,7 @@
         </is>
       </c>
       <c r="G65" t="n">
-        <v>5.84</v>
+        <v>11.12</v>
       </c>
     </row>
     <row r="66">
@@ -2731,7 +2740,7 @@
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>On-Demand</t>
+          <t>Spot</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
@@ -2745,7 +2754,7 @@
         </is>
       </c>
       <c r="G66" t="n">
-        <v>11.12</v>
+        <v>5.25</v>
       </c>
     </row>
     <row r="67">
@@ -2761,12 +2770,12 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>B200</t>
+          <t>H200</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Spot</t>
+          <t>On-Demand</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
@@ -2780,7 +2789,7 @@
         </is>
       </c>
       <c r="G67" t="n">
-        <v>5.25</v>
+        <v>7.09</v>
       </c>
     </row>
     <row r="68">
@@ -2801,7 +2810,7 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>On-Demand</t>
+          <t>Spot</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
@@ -2815,7 +2824,7 @@
         </is>
       </c>
       <c r="G68" t="n">
-        <v>7.09</v>
+        <v>3.35</v>
       </c>
     </row>
     <row r="69">
@@ -2831,12 +2840,12 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>H200</t>
+          <t>A100</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Spot</t>
+          <t>On-Demand</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
@@ -2850,7 +2859,7 @@
         </is>
       </c>
       <c r="G69" t="n">
-        <v>3.35</v>
+        <v>1.43</v>
       </c>
     </row>
     <row r="70">
@@ -2871,7 +2880,7 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>On-Demand</t>
+          <t>Spot</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
@@ -2885,7 +2894,7 @@
         </is>
       </c>
       <c r="G70" t="n">
-        <v>1.43</v>
+        <v>1.2</v>
       </c>
     </row>
     <row r="71">
@@ -2896,17 +2905,17 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Spheron</t>
+          <t>Hyperbolic</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>A100</t>
+          <t>B200</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Spot</t>
+          <t>N/A</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
@@ -2920,7 +2929,7 @@
         </is>
       </c>
       <c r="G71" t="n">
-        <v>1.38</v>
+        <v>5.99</v>
       </c>
     </row>
     <row r="72">
@@ -2936,7 +2945,7 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>B200</t>
+          <t>H200</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
@@ -2955,7 +2964,7 @@
         </is>
       </c>
       <c r="G72" t="n">
-        <v>5.99</v>
+        <v>3.99</v>
       </c>
     </row>
     <row r="73">
@@ -2966,12 +2975,12 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Hyperbolic</t>
+          <t>DeepInfra</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>H200</t>
+          <t>B300</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
@@ -2990,7 +2999,7 @@
         </is>
       </c>
       <c r="G73" t="n">
-        <v>3.99</v>
+        <v>5.89</v>
       </c>
     </row>
     <row r="74">
@@ -3006,7 +3015,7 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>B300</t>
+          <t>B200</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
@@ -3025,7 +3034,7 @@
         </is>
       </c>
       <c r="G74" t="n">
-        <v>5.89</v>
+        <v>4.89</v>
       </c>
     </row>
     <row r="75">
@@ -3041,7 +3050,7 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>B200</t>
+          <t>H200</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -3060,7 +3069,7 @@
         </is>
       </c>
       <c r="G75" t="n">
-        <v>4.89</v>
+        <v>3.49</v>
       </c>
     </row>
     <row r="76">
@@ -3076,7 +3085,7 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>H200</t>
+          <t>A100</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
@@ -3095,7 +3104,7 @@
         </is>
       </c>
       <c r="G76" t="n">
-        <v>3.49</v>
+        <v>1.49</v>
       </c>
     </row>
     <row r="77">
@@ -3106,12 +3115,12 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>DeepInfra</t>
+          <t>Fireworks.ai</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>A100</t>
+          <t>GB300</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -3130,7 +3139,7 @@
         </is>
       </c>
       <c r="G77" t="n">
-        <v>1.49</v>
+        <v>20</v>
       </c>
     </row>
     <row r="78">
@@ -3146,7 +3155,7 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>GB300</t>
+          <t>B300</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -3165,7 +3174,7 @@
         </is>
       </c>
       <c r="G78" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
     </row>
     <row r="79">
@@ -3181,7 +3190,7 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>B300</t>
+          <t>B200</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -3200,7 +3209,7 @@
         </is>
       </c>
       <c r="G79" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
     </row>
     <row r="80">
@@ -3216,7 +3225,7 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>B200</t>
+          <t>H200</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -3235,7 +3244,7 @@
         </is>
       </c>
       <c r="G80" t="n">
-        <v>13</v>
+        <v>8</v>
       </c>
     </row>
     <row r="81">
@@ -3246,17 +3255,17 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Fireworks.ai</t>
+          <t>Astra Intellectus</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>H200</t>
+          <t>GB300</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>N/A</t>
+          <t>Reserve</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
@@ -3270,7 +3279,7 @@
         </is>
       </c>
       <c r="G81" t="n">
-        <v>8</v>
+        <v>6.25</v>
       </c>
     </row>
     <row r="82">
@@ -3286,7 +3295,7 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>GB300</t>
+          <t>B300</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
@@ -3305,7 +3314,7 @@
         </is>
       </c>
       <c r="G82" t="n">
-        <v>6.25</v>
+        <v>5.45</v>
       </c>
     </row>
     <row r="83">
@@ -3316,17 +3325,17 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Astra Intellectus</t>
+          <t>Verda</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>B300</t>
+          <t>GB300</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Reserve</t>
+          <t>On-Demand</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
@@ -3340,7 +3349,7 @@
         </is>
       </c>
       <c r="G83" t="n">
-        <v>5.45</v>
+        <v>12.55</v>
       </c>
     </row>
     <row r="84">
@@ -3351,17 +3360,17 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Astra Intellectus</t>
+          <t>Verda</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>H200</t>
+          <t>GB300</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Reserve</t>
+          <t>Spot</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
@@ -3373,6 +3382,9 @@
         <is>
           <t>N/A</t>
         </is>
+      </c>
+      <c r="G84" t="n">
+        <v>6.273</v>
       </c>
     </row>
     <row r="85">
@@ -3388,7 +3400,7 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>GB300</t>
+          <t>B300</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -3407,7 +3419,7 @@
         </is>
       </c>
       <c r="G85" t="n">
-        <v>12.55</v>
+        <v>10.91</v>
       </c>
     </row>
     <row r="86">
@@ -3423,7 +3435,7 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>GB300</t>
+          <t>B300</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -3442,7 +3454,7 @@
         </is>
       </c>
       <c r="G86" t="n">
-        <v>6.273</v>
+        <v>5.455</v>
       </c>
     </row>
     <row r="87">
@@ -3458,7 +3470,7 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>B300</t>
+          <t>B200</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -3477,7 +3489,7 @@
         </is>
       </c>
       <c r="G87" t="n">
-        <v>10.91</v>
+        <v>8.523</v>
       </c>
     </row>
     <row r="88">
@@ -3493,7 +3505,7 @@
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>B300</t>
+          <t>B200</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -3512,7 +3524,7 @@
         </is>
       </c>
       <c r="G88" t="n">
-        <v>5.455</v>
+        <v>4.262</v>
       </c>
     </row>
     <row r="89">
@@ -3528,7 +3540,7 @@
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>B200</t>
+          <t>H200</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -3547,7 +3559,7 @@
         </is>
       </c>
       <c r="G89" t="n">
-        <v>8.523</v>
+        <v>6.006</v>
       </c>
     </row>
     <row r="90">
@@ -3563,7 +3575,7 @@
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>B200</t>
+          <t>H200</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
@@ -3582,7 +3594,7 @@
         </is>
       </c>
       <c r="G90" t="n">
-        <v>4.262</v>
+        <v>3.003</v>
       </c>
     </row>
     <row r="91">
@@ -3598,7 +3610,7 @@
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>H200</t>
+          <t>A100</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -3617,7 +3629,7 @@
         </is>
       </c>
       <c r="G91" t="n">
-        <v>6.006</v>
+        <v>2.16</v>
       </c>
     </row>
     <row r="92">
@@ -3633,7 +3645,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>H200</t>
+          <t>A100</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
@@ -3652,76 +3664,6 @@
         </is>
       </c>
       <c r="G92" t="n">
-        <v>3.003</v>
-      </c>
-    </row>
-    <row r="93">
-      <c r="A93" t="inlineStr">
-        <is>
-          <t>20261026</t>
-        </is>
-      </c>
-      <c r="B93" t="inlineStr">
-        <is>
-          <t>Verda</t>
-        </is>
-      </c>
-      <c r="C93" t="inlineStr">
-        <is>
-          <t>A100</t>
-        </is>
-      </c>
-      <c r="D93" t="inlineStr">
-        <is>
-          <t>On-Demand</t>
-        </is>
-      </c>
-      <c r="E93" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F93" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G93" t="n">
-        <v>2.16</v>
-      </c>
-    </row>
-    <row r="94">
-      <c r="A94" t="inlineStr">
-        <is>
-          <t>20261026</t>
-        </is>
-      </c>
-      <c r="B94" t="inlineStr">
-        <is>
-          <t>Verda</t>
-        </is>
-      </c>
-      <c r="C94" t="inlineStr">
-        <is>
-          <t>A100</t>
-        </is>
-      </c>
-      <c r="D94" t="inlineStr">
-        <is>
-          <t>Spot</t>
-        </is>
-      </c>
-      <c r="E94" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="F94" t="inlineStr">
-        <is>
-          <t>N/A</t>
-        </is>
-      </c>
-      <c r="G94" t="n">
         <v>1.08</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add October historical GPU price dataset
Co-authored-by: DanielWang2029 <DanielWang2029@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/output/gpu_prices_20261026.xlsx
+++ b/output/gpu_prices_20261026.xlsx
@@ -1039,7 +1039,7 @@
         </is>
       </c>
       <c r="G17" t="n">
-        <v>5.5</v>
+        <v>5.2</v>
       </c>
     </row>
     <row r="18">
@@ -1074,7 +1074,7 @@
         </is>
       </c>
       <c r="G18" t="n">
-        <v>9.49</v>
+        <v>9.19</v>
       </c>
     </row>
     <row r="19">
@@ -1109,7 +1109,7 @@
         </is>
       </c>
       <c r="G19" t="n">
-        <v>2.7</v>
+        <v>2.4</v>
       </c>
     </row>
     <row r="20">
@@ -1144,7 +1144,7 @@
         </is>
       </c>
       <c r="G20" t="n">
-        <v>6.2</v>
+        <v>6.5</v>
       </c>
     </row>
     <row r="21">
@@ -1179,7 +1179,7 @@
         </is>
       </c>
       <c r="G21" t="n">
-        <v>5.09</v>
+        <v>4.79</v>
       </c>
     </row>
     <row r="22">
@@ -1459,7 +1459,7 @@
         </is>
       </c>
       <c r="G29" t="n">
-        <v>3.68</v>
+        <v>3.99</v>
       </c>
     </row>
     <row r="30">
@@ -1564,7 +1564,7 @@
         </is>
       </c>
       <c r="G32" t="n">
-        <v>1.77</v>
+        <v>1.54</v>
       </c>
     </row>
     <row r="33">
@@ -2719,7 +2719,7 @@
         </is>
       </c>
       <c r="G65" t="n">
-        <v>11.12</v>
+        <v>10.39</v>
       </c>
     </row>
     <row r="66">
@@ -2754,7 +2754,7 @@
         </is>
       </c>
       <c r="G66" t="n">
-        <v>5.25</v>
+        <v>5.22</v>
       </c>
     </row>
     <row r="67">
@@ -2894,7 +2894,7 @@
         </is>
       </c>
       <c r="G70" t="n">
-        <v>1.2</v>
+        <v>1.19</v>
       </c>
     </row>
     <row r="71">

</xml_diff>